<commit_message>
Moved enum mapping for institution_type from maps tab to enums tab
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FBB2A9-AF9D-0442-A2AB-565E65037983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA7715B2-6530-D44C-B85D-24D37FC76ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" activeTab="6" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2812" uniqueCount="809">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2769" uniqueCount="811">
   <si>
     <t>Reporter</t>
   </si>
@@ -2529,6 +2529,12 @@
   </si>
   <si>
     <t>sample_collect_date + '/!/' + sample_collect_time + '/!/' + time_zone</t>
+  </si>
+  <si>
+    <t>vs_institution_type</t>
+  </si>
+  <si>
+    <t>{{institution_type}}</t>
   </si>
 </sst>
 </file>
@@ -2710,7 +2716,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -2787,9 +2793,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -13959,7 +13962,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}">
-  <dimension ref="A1:K102"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -15352,7 +15355,7 @@
     </row>
     <row r="79" spans="1:8" s="23" customFormat="1">
       <c r="A79" s="23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B79" s="23" t="s">
         <v>630</v>
@@ -15392,7 +15395,7 @@
       </c>
       <c r="H80" s="39"/>
     </row>
-    <row r="81" spans="1:10" s="23" customFormat="1">
+    <row r="81" spans="1:8" s="23" customFormat="1">
       <c r="A81" s="23" t="b">
         <v>1</v>
       </c>
@@ -15413,7 +15416,7 @@
       </c>
       <c r="H81" s="39"/>
     </row>
-    <row r="82" spans="1:10" s="23" customFormat="1">
+    <row r="82" spans="1:8" s="23" customFormat="1">
       <c r="A82" s="23" t="b">
         <v>1</v>
       </c>
@@ -15434,7 +15437,7 @@
       </c>
       <c r="H82" s="39"/>
     </row>
-    <row r="83" spans="1:10" s="23" customFormat="1" ht="17" customHeight="1">
+    <row r="83" spans="1:8" s="23" customFormat="1" ht="17" customHeight="1">
       <c r="A83" s="23" t="b">
         <v>1</v>
       </c>
@@ -15455,7 +15458,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="84" spans="1:10" s="23" customFormat="1">
+    <row r="84" spans="1:8" s="23" customFormat="1">
       <c r="A84" s="23" t="b">
         <v>1</v>
       </c>
@@ -15477,7 +15480,7 @@
       </c>
       <c r="H84" s="39"/>
     </row>
-    <row r="85" spans="1:10" s="23" customFormat="1">
+    <row r="85" spans="1:8" s="23" customFormat="1">
       <c r="A85" s="23" t="b">
         <v>1</v>
       </c>
@@ -15498,7 +15501,7 @@
       </c>
       <c r="H85" s="39"/>
     </row>
-    <row r="86" spans="1:10" s="23" customFormat="1">
+    <row r="86" spans="1:8" s="23" customFormat="1">
       <c r="A86" s="23" t="b">
         <v>1</v>
       </c>
@@ -15519,393 +15522,25 @@
       </c>
       <c r="H86" s="39"/>
     </row>
-    <row r="87" spans="1:10" s="17" customFormat="1" ht="17" customHeight="1">
-      <c r="A87" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B87" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C87" s="23" t="s">
+    <row r="87" spans="1:8">
+      <c r="A87" t="b">
+        <v>1</v>
+      </c>
+      <c r="B87" t="s">
+        <v>630</v>
+      </c>
+      <c r="C87" t="s">
         <v>15</v>
       </c>
-      <c r="D87" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="E87" s="23" t="s">
+      <c r="E87" t="s">
         <v>76</v>
       </c>
-      <c r="F87" s="23" t="s">
+      <c r="F87" t="s">
         <v>100</v>
       </c>
-      <c r="G87" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="H87" s="39"/>
-      <c r="I87" s="23"/>
-      <c r="J87" s="23"/>
-    </row>
-    <row r="88" spans="1:10" s="23" customFormat="1">
-      <c r="A88" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B88" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C88" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D88" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="E88" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F88" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G88" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="H88" s="39"/>
-    </row>
-    <row r="89" spans="1:10" s="23" customFormat="1">
-      <c r="A89" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B89" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C89" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D89" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="E89" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F89" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G89" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="H89" s="39"/>
-    </row>
-    <row r="90" spans="1:10" s="23" customFormat="1">
-      <c r="A90" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B90" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C90" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D90" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="E90" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F90" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G90" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="H90" s="39"/>
-    </row>
-    <row r="91" spans="1:10" s="23" customFormat="1">
-      <c r="A91" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B91" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C91" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D91" s="30" t="s">
-        <v>88</v>
-      </c>
-      <c r="E91" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F91" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G91" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="H91" s="39"/>
-    </row>
-    <row r="92" spans="1:10" s="23" customFormat="1">
-      <c r="A92" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B92" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C92" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D92" s="28" t="s">
-        <v>89</v>
-      </c>
-      <c r="E92" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F92" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G92" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="H92" s="39"/>
-    </row>
-    <row r="93" spans="1:10" s="23" customFormat="1">
-      <c r="A93" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B93" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C93" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D93" s="28" t="s">
-        <v>90</v>
-      </c>
-      <c r="E93" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F93" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G93" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="H93" s="39"/>
-    </row>
-    <row r="94" spans="1:10" s="23" customFormat="1">
-      <c r="A94" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B94" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C94" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D94" s="29" t="s">
-        <v>91</v>
-      </c>
-      <c r="E94" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F94" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G94" s="23" t="s">
-        <v>109</v>
-      </c>
-      <c r="H94" s="39"/>
-    </row>
-    <row r="95" spans="1:10" s="23" customFormat="1">
-      <c r="A95" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B95" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C95" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D95" s="29" t="s">
-        <v>92</v>
-      </c>
-      <c r="E95" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F95" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G95" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="H95" s="39"/>
-    </row>
-    <row r="96" spans="1:10" s="23" customFormat="1">
-      <c r="A96" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B96" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C96" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D96" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="E96" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F96" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G96" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="H96" s="39"/>
-    </row>
-    <row r="97" spans="1:11" s="23" customFormat="1">
-      <c r="A97" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B97" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C97" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D97" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="E97" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F97" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G97" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="H97" s="39"/>
-    </row>
-    <row r="98" spans="1:11" s="23" customFormat="1">
-      <c r="A98" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B98" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C98" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D98" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="E98" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F98" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G98" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="H98" s="39"/>
-    </row>
-    <row r="99" spans="1:11" s="23" customFormat="1">
-      <c r="A99" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B99" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C99" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D99" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="E99" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F99" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G99" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="H99" s="39"/>
-    </row>
-    <row r="100" spans="1:11" s="23" customFormat="1">
-      <c r="A100" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B100" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C100" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D100" s="28" t="s">
-        <v>97</v>
-      </c>
-      <c r="E100" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F100" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G100" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="H100" s="39"/>
-    </row>
-    <row r="101" spans="1:11" s="23" customFormat="1">
-      <c r="A101" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B101" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C101" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D101" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="E101" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F101" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G101" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="H101" s="39"/>
-    </row>
-    <row r="102" spans="1:11" s="23" customFormat="1">
-      <c r="A102" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B102" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="C102" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="D102" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="E102" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="F102" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G102" s="37" t="s">
-        <v>530</v>
-      </c>
-      <c r="H102" s="42"/>
-      <c r="I102" s="25"/>
-      <c r="K102" s="37"/>
+      <c r="G87" t="s">
+        <v>810</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20744,7 +20379,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC10C3F-0C27-5546-8767-E60C7CACEA9D}">
-  <dimension ref="A1:J191"/>
+  <dimension ref="A1:J208"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
@@ -23386,6 +23021,230 @@
       </c>
       <c r="I191" t="s">
         <v>532</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9">
+      <c r="A193" t="b">
+        <v>1</v>
+      </c>
+      <c r="D193" t="s">
+        <v>809</v>
+      </c>
+      <c r="E193" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="I193" s="23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9">
+      <c r="A194" t="b">
+        <v>1</v>
+      </c>
+      <c r="D194" t="s">
+        <v>809</v>
+      </c>
+      <c r="E194" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="I194" s="23" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9">
+      <c r="A195" t="b">
+        <v>1</v>
+      </c>
+      <c r="D195" t="s">
+        <v>809</v>
+      </c>
+      <c r="E195" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="I195" s="23" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9">
+      <c r="A196" t="b">
+        <v>1</v>
+      </c>
+      <c r="D196" t="s">
+        <v>809</v>
+      </c>
+      <c r="E196" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="I196" s="23" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9">
+      <c r="A197" t="b">
+        <v>1</v>
+      </c>
+      <c r="D197" t="s">
+        <v>809</v>
+      </c>
+      <c r="E197" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="I197" s="23" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9">
+      <c r="A198" t="b">
+        <v>1</v>
+      </c>
+      <c r="D198" t="s">
+        <v>809</v>
+      </c>
+      <c r="E198" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="I198" s="23" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9">
+      <c r="A199" t="b">
+        <v>1</v>
+      </c>
+      <c r="D199" t="s">
+        <v>809</v>
+      </c>
+      <c r="E199" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="I199" s="23" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9">
+      <c r="A200" t="b">
+        <v>1</v>
+      </c>
+      <c r="D200" t="s">
+        <v>809</v>
+      </c>
+      <c r="E200" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="I200" s="23" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9">
+      <c r="A201" t="b">
+        <v>1</v>
+      </c>
+      <c r="D201" t="s">
+        <v>809</v>
+      </c>
+      <c r="E201" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="I201" s="23" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9">
+      <c r="A202" t="b">
+        <v>1</v>
+      </c>
+      <c r="D202" t="s">
+        <v>809</v>
+      </c>
+      <c r="E202" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="I202" s="23" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9">
+      <c r="A203" t="b">
+        <v>1</v>
+      </c>
+      <c r="D203" t="s">
+        <v>809</v>
+      </c>
+      <c r="E203" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="I203" s="23" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9">
+      <c r="A204" t="b">
+        <v>1</v>
+      </c>
+      <c r="D204" t="s">
+        <v>809</v>
+      </c>
+      <c r="E204" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="I204" s="23" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9">
+      <c r="A205" t="b">
+        <v>1</v>
+      </c>
+      <c r="D205" t="s">
+        <v>809</v>
+      </c>
+      <c r="E205" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="I205" s="23" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9">
+      <c r="A206" t="b">
+        <v>1</v>
+      </c>
+      <c r="D206" t="s">
+        <v>809</v>
+      </c>
+      <c r="E206" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="I206" s="23" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9">
+      <c r="A207" t="b">
+        <v>1</v>
+      </c>
+      <c r="D207" t="s">
+        <v>809</v>
+      </c>
+      <c r="E207" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="I207" s="23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9">
+      <c r="A208" t="b">
+        <v>1</v>
+      </c>
+      <c r="D208" t="s">
+        <v>809</v>
+      </c>
+      <c r="E208" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="I208" s="37" t="s">
+        <v>530</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added selectors for rec_eff_percent in wide_measures: Mapping is different for ODM v2 and v3
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7EBD55-827F-6243-BD48-0D9FEE1B89C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18857A13-B1CB-E84E-BE47-72AF98C007BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" activeTab="1" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">enums!$A$1:$J$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$K$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'maps original'!$A$1:$L$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide_measures!$A$1:$S$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide_measures!$A$1:$T$25</definedName>
     <definedName name="partID">[1]parts!$A:$A</definedName>
     <definedName name="partLabel">[1]parts!$B:$B</definedName>
   </definedNames>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2908" uniqueCount="815">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2921" uniqueCount="820">
   <si>
     <t>Reporter</t>
   </si>
@@ -2281,9 +2281,6 @@
   </si>
   <si>
     <t>&lt;ignore&gt;</t>
-  </si>
-  <si>
-    <t>stepID_value</t>
   </si>
   <si>
     <t>value_expr</t>
@@ -2547,6 +2544,24 @@
   </si>
   <si>
     <t>extractRecov</t>
+  </si>
+  <si>
+    <t>summ_value</t>
+  </si>
+  <si>
+    <t>odm&gt;=3</t>
+  </si>
+  <si>
+    <t>odm&lt;3</t>
+  </si>
+  <si>
+    <t>percRec</t>
+  </si>
+  <si>
+    <t>selectors</t>
+  </si>
+  <si>
+    <t>null</t>
   </si>
 </sst>
 </file>
@@ -14148,7 +14163,7 @@
         <v>713</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -14162,7 +14177,7 @@
         <v>713</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
@@ -14176,7 +14191,7 @@
         <v>713</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
@@ -14190,7 +14205,7 @@
         <v>713</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -14204,7 +14219,7 @@
         <v>713</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -14218,7 +14233,7 @@
         <v>713</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -14449,10 +14464,10 @@
         <v>114</v>
       </c>
       <c r="F28" s="25" t="s">
+        <v>752</v>
+      </c>
+      <c r="H28" s="34" t="s">
         <v>753</v>
-      </c>
-      <c r="H28" s="34" t="s">
-        <v>754</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -14569,7 +14584,7 @@
         <v>708</v>
       </c>
       <c r="F36" s="25" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
@@ -14604,7 +14619,7 @@
         <v>708</v>
       </c>
       <c r="F38" s="25" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
@@ -14618,7 +14633,7 @@
         <v>708</v>
       </c>
       <c r="F39" s="25" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -14632,7 +14647,7 @@
         <v>708</v>
       </c>
       <c r="F40" s="25" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
@@ -14646,7 +14661,7 @@
         <v>708</v>
       </c>
       <c r="F41" s="25" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
@@ -14799,7 +14814,7 @@
         <v>472</v>
       </c>
       <c r="F51" s="25" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G51" s="25" t="s">
         <v>689</v>
@@ -14919,7 +14934,7 @@
         <v>119</v>
       </c>
       <c r="H59" s="36" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -14937,10 +14952,10 @@
         <v>137</v>
       </c>
       <c r="H60" s="36" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="J60" s="25" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
@@ -14960,7 +14975,7 @@
         <v>144</v>
       </c>
       <c r="H61" s="33" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
@@ -15390,7 +15405,7 @@
         <v>83</v>
       </c>
       <c r="H83" s="36" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.2">
@@ -15471,7 +15486,7 @@
         <v>100</v>
       </c>
       <c r="G87" s="25" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
   </sheetData>
@@ -15482,30 +15497,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39AC7DD-3F73-2C47-925D-21E5B4EBE6FC}">
-  <dimension ref="A1:S26"/>
+  <dimension ref="A1:T28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="25"/>
     <col min="2" max="2" width="13" style="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.1640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" style="25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.33203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.83203125" style="25" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="83.6640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="16" max="18" width="21.83203125" style="25" customWidth="1"/>
-    <col min="19" max="19" width="27.6640625" style="25" customWidth="1"/>
-    <col min="20" max="16384" width="10.83203125" style="25"/>
+    <col min="3" max="3" width="13" style="25" customWidth="1"/>
+    <col min="4" max="4" width="21.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" style="25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" style="25" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.33203125" style="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.83203125" style="25" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" style="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22" style="25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="83.6640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.1640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="17" max="19" width="21.83203125" style="25" customWidth="1"/>
+    <col min="20" max="20" width="27.6640625" style="25" customWidth="1"/>
+    <col min="21" max="16384" width="10.83203125" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="31" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
         <v>651</v>
       </c>
@@ -15513,863 +15529,904 @@
         <v>614</v>
       </c>
       <c r="C1" s="31" t="s">
+        <v>818</v>
+      </c>
+      <c r="D1" s="31" t="s">
         <v>616</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="E1" s="31" t="s">
         <v>617</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="F1" s="31" t="s">
         <v>618</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="G1" s="31" t="s">
         <v>620</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="H1" s="31" t="s">
         <v>667</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="I1" s="31" t="s">
         <v>732</v>
       </c>
-      <c r="I1" s="31" t="s">
+      <c r="J1" s="31" t="s">
+        <v>750</v>
+      </c>
+      <c r="K1" s="32" t="s">
+        <v>724</v>
+      </c>
+      <c r="L1" s="32" t="s">
+        <v>725</v>
+      </c>
+      <c r="M1" s="32" t="s">
+        <v>727</v>
+      </c>
+      <c r="N1" s="32" t="s">
+        <v>734</v>
+      </c>
+      <c r="O1" s="32" t="s">
+        <v>728</v>
+      </c>
+      <c r="P1" s="32" t="s">
+        <v>729</v>
+      </c>
+      <c r="Q1" s="31" t="s">
         <v>751</v>
       </c>
-      <c r="J1" s="32" t="s">
-        <v>724</v>
-      </c>
-      <c r="K1" s="32" t="s">
-        <v>725</v>
-      </c>
-      <c r="L1" s="32" t="s">
-        <v>727</v>
-      </c>
-      <c r="M1" s="32" t="s">
+      <c r="R1" s="31" t="s">
+        <v>744</v>
+      </c>
+      <c r="S1" s="31" t="s">
         <v>735</v>
       </c>
-      <c r="N1" s="32" t="s">
-        <v>728</v>
-      </c>
-      <c r="O1" s="32" t="s">
-        <v>729</v>
-      </c>
-      <c r="P1" s="31" t="s">
-        <v>752</v>
-      </c>
-      <c r="Q1" s="31" t="s">
-        <v>745</v>
-      </c>
-      <c r="R1" s="31" t="s">
-        <v>736</v>
-      </c>
-      <c r="S1" s="32" t="s">
+      <c r="T1" s="32" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B2" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="D2" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="F2" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F2" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J2" s="25" t="s">
-        <v>799</v>
+      <c r="G2" s="25" t="s">
+        <v>630</v>
       </c>
       <c r="K2" s="25" t="s">
+        <v>798</v>
+      </c>
+      <c r="L2" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="M2" s="25" t="s">
-        <v>771</v>
-      </c>
       <c r="N2" s="25" t="s">
+        <v>770</v>
+      </c>
+      <c r="O2" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="O2" s="25" t="s">
+      <c r="P2" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B3" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="D3" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="F3" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F3" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J3" s="25" t="s">
+      <c r="G3" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K3" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="K3" s="25" t="s">
+      <c r="L3" s="25" t="s">
         <v>165</v>
       </c>
-      <c r="L3" s="25" t="s">
+      <c r="M3" s="25" t="s">
         <v>633</v>
       </c>
-      <c r="N3" s="25" t="s">
+      <c r="O3" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="O3" s="25" t="s">
+      <c r="P3" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B4" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="D4" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="F4" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J4" s="25" t="s">
+      <c r="G4" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K4" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="K4" s="25" t="s">
+      <c r="L4" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="L4" s="25" t="s">
+      <c r="M4" s="25" t="s">
         <v>632</v>
       </c>
-      <c r="N4" s="25" t="s">
+      <c r="O4" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="O4" s="25" t="s">
+      <c r="P4" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B5" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="D5" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="F5" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F5" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J5" s="25" t="s">
+      <c r="G5" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K5" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="K5" s="25" t="s">
+      <c r="L5" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="L5" s="25" t="s">
+      <c r="M5" s="25" t="s">
         <v>645</v>
       </c>
-      <c r="N5" s="25" t="s">
+      <c r="O5" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="O5" s="25" t="s">
+      <c r="P5" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B6" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="D6" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="F6" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F6" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J6" s="25" t="s">
+      <c r="G6" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K6" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="K6" s="25" t="s">
+      <c r="L6" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="M6" s="25" t="s">
         <v>643</v>
       </c>
-      <c r="N6" s="25" t="s">
+      <c r="O6" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="O6" s="25" t="s">
+      <c r="P6" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B7" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="D7" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="F7" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F7" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J7" s="25" t="s">
+      <c r="G7" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K7" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="K7" s="25" t="s">
+      <c r="L7" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="L7" s="25" t="s">
+      <c r="M7" s="25" t="s">
         <v>646</v>
       </c>
-      <c r="N7" s="25" t="s">
-        <v>756</v>
-      </c>
       <c r="O7" s="25" t="s">
+        <v>755</v>
+      </c>
+      <c r="P7" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B8" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="D8" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="F8" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F8" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J8" s="25" t="s">
-        <v>799</v>
+      <c r="G8" s="25" t="s">
+        <v>630</v>
       </c>
       <c r="K8" s="25" t="s">
+        <v>798</v>
+      </c>
+      <c r="L8" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="M8" s="25" t="s">
-        <v>770</v>
-      </c>
       <c r="N8" s="25" t="s">
+        <v>769</v>
+      </c>
+      <c r="O8" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="O8" s="25" t="s">
+      <c r="P8" s="25" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B9" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C9" s="25" t="s">
+      <c r="D9" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="F9" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F9" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J9" s="25" t="s">
+      <c r="G9" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K9" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="K9" s="25" t="s">
+      <c r="L9" s="25" t="s">
         <v>624</v>
       </c>
-      <c r="L9" s="25" t="s">
+      <c r="M9" s="25" t="s">
         <v>649</v>
       </c>
-      <c r="N9" s="25" t="s">
+      <c r="O9" s="25" t="s">
         <v>628</v>
       </c>
-      <c r="O9" s="25" t="s">
+      <c r="P9" s="25" t="s">
         <v>156</v>
       </c>
-      <c r="P9" s="25" t="s">
+      <c r="Q9" s="25" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A10" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G10" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K10" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L10" s="25" t="s">
+        <v>623</v>
+      </c>
+      <c r="M10" s="25" t="s">
+        <v>648</v>
+      </c>
+      <c r="O10" s="25" t="s">
+        <v>627</v>
+      </c>
+      <c r="P10" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q10" s="25" t="s">
         <v>740</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A10" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="E10" s="25" t="s">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A11" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J10" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K10" s="25" t="s">
-        <v>623</v>
-      </c>
-      <c r="L10" s="25" t="s">
-        <v>648</v>
-      </c>
-      <c r="N10" s="25" t="s">
-        <v>627</v>
-      </c>
-      <c r="O10" s="25" t="s">
+      <c r="G11" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K11" s="25" t="s">
+        <v>798</v>
+      </c>
+      <c r="L11" s="25" t="s">
+        <v>160</v>
+      </c>
+      <c r="N11" s="25" t="s">
+        <v>768</v>
+      </c>
+      <c r="O11" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="P11" s="25" t="s">
         <v>156</v>
       </c>
-      <c r="P10" s="25" t="s">
-        <v>741</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" s="25" t="s">
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A12" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="F12" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F11" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J11" s="25" t="s">
-        <v>799</v>
-      </c>
-      <c r="K11" s="25" t="s">
-        <v>160</v>
-      </c>
-      <c r="M11" s="25" t="s">
-        <v>769</v>
-      </c>
-      <c r="N11" s="25" t="s">
-        <v>161</v>
-      </c>
-      <c r="O11" s="25" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A12" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="E12" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F12" s="25" t="str">
+      <c r="G12" s="25" t="str">
         <f>"true"</f>
         <v>true</v>
       </c>
-      <c r="J12" s="25" t="s">
-        <v>799</v>
-      </c>
       <c r="K12" s="25" t="s">
+        <v>798</v>
+      </c>
+      <c r="L12" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="L12" s="25" t="s">
+      <c r="M12" s="25" t="s">
         <v>631</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B13" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="D13" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="E13" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="F13" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F13" s="25" t="str">
+      <c r="G13" s="25" t="str">
         <f>"false"</f>
         <v>false</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="b">
         <v>1</v>
       </c>
       <c r="B14" s="25" t="s">
         <v>615</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="D14" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="E14" s="25" t="s">
         <v>720</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="F14" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F14" s="25" t="s">
+      <c r="G14" s="25" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A15" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G15" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K15" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L15" s="25" t="s">
+        <v>582</v>
+      </c>
+      <c r="M15" s="25" t="s">
+        <v>647</v>
+      </c>
+      <c r="O15" s="25" t="s">
+        <v>626</v>
+      </c>
+      <c r="P15" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q15" s="25" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A16" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G16" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="J16" s="25" t="s">
+        <v>738</v>
+      </c>
+      <c r="K16" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L16" s="25" t="s">
+        <v>625</v>
+      </c>
+      <c r="M16" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="O16" s="25" t="s">
+        <v>629</v>
+      </c>
+      <c r="P16" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q16" s="25" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A17" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K17" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L17" s="25" t="s">
+        <v>622</v>
+      </c>
+      <c r="N17" s="25" t="s">
+        <v>785</v>
+      </c>
+      <c r="O17" s="25" t="s">
+        <v>626</v>
+      </c>
+      <c r="P17" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q17" s="25" t="s">
+        <v>743</v>
+      </c>
+      <c r="R17" s="25" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A18" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F18" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G18" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K18" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L18" s="25" t="s">
+        <v>622</v>
+      </c>
+      <c r="N18" s="25" t="s">
+        <v>788</v>
+      </c>
+      <c r="O18" s="25" t="s">
+        <v>626</v>
+      </c>
+      <c r="P18" s="25" t="s">
+        <v>577</v>
+      </c>
+      <c r="Q18" s="25" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A19" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="F19" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K19" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L19" s="25" t="s">
+        <v>622</v>
+      </c>
+      <c r="N19" s="25" t="s">
+        <v>787</v>
+      </c>
+      <c r="O19" s="25" t="s">
+        <v>626</v>
+      </c>
+      <c r="P19" s="25" t="s">
+        <v>578</v>
+      </c>
+      <c r="Q19" s="25" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A20" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G20" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K20" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L20" s="25" t="s">
+        <v>622</v>
+      </c>
+      <c r="N20" s="25" t="s">
+        <v>786</v>
+      </c>
+      <c r="O20" s="25" t="s">
+        <v>626</v>
+      </c>
+      <c r="P20" s="25" t="s">
+        <v>812</v>
+      </c>
+      <c r="Q20" s="25" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A21" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K21" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L21" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="M21" s="25" t="s">
+        <v>642</v>
+      </c>
+      <c r="O21" s="25" t="s">
+        <v>169</v>
+      </c>
+      <c r="P21" s="25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A22" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K22" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L22" s="25" t="s">
+        <v>167</v>
+      </c>
+      <c r="M22" s="25" t="s">
+        <v>621</v>
+      </c>
+      <c r="S22" s="25" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A23" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="F23" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G23" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K23" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L23" s="25" t="s">
+        <v>566</v>
+      </c>
+      <c r="M23" s="25" t="s">
+        <v>640</v>
+      </c>
+      <c r="O23" s="25" t="s">
+        <v>567</v>
+      </c>
+      <c r="P23" s="25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A24" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G24" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K24" s="25" t="s">
+        <v>798</v>
+      </c>
+      <c r="L24" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="M24" s="26"/>
+      <c r="N24" s="26" t="s">
         <v>767</v>
       </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A15" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B15" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C15" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="E15" s="25" t="s">
+      <c r="O24" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="P24" s="26" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A25" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="F25" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F15" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J15" s="25" t="s">
+      <c r="G25" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K25" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="K15" s="25" t="s">
-        <v>582</v>
-      </c>
-      <c r="L15" s="25" t="s">
-        <v>647</v>
-      </c>
-      <c r="N15" s="25" t="s">
-        <v>626</v>
-      </c>
-      <c r="O15" s="25" t="s">
+      <c r="L25" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="M25" s="25" t="s">
+        <v>644</v>
+      </c>
+      <c r="O25" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="P25" s="25" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A27" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B27" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>816</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K27" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="L27" s="25" t="s">
+        <v>817</v>
+      </c>
+      <c r="N27" s="25" t="s">
+        <v>784</v>
+      </c>
+      <c r="O27" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="P27" s="25" t="s">
         <v>156</v>
       </c>
-      <c r="P15" s="25" t="s">
-        <v>742</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A16" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B16" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C16" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="E16" s="25" t="s">
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A28" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B28" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>815</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="F28" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F16" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="I16" s="25" t="s">
-        <v>739</v>
-      </c>
-      <c r="J16" s="25" t="s">
+      <c r="G28" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="K28" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="K16" s="25" t="s">
-        <v>625</v>
-      </c>
-      <c r="L16" s="25" t="s">
-        <v>650</v>
-      </c>
-      <c r="N16" s="25" t="s">
-        <v>629</v>
-      </c>
-      <c r="O16" s="25" t="s">
+      <c r="L28" s="25" t="s">
+        <v>813</v>
+      </c>
+      <c r="N28" s="25" t="s">
+        <v>784</v>
+      </c>
+      <c r="O28" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="P28" s="25" t="s">
         <v>156</v>
       </c>
-      <c r="P16" s="25" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="E17" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F17" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J17" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K17" s="25" t="s">
-        <v>622</v>
-      </c>
-      <c r="M17" s="25" t="s">
-        <v>786</v>
-      </c>
-      <c r="N17" s="25" t="s">
-        <v>626</v>
-      </c>
-      <c r="O17" s="25" t="s">
-        <v>156</v>
-      </c>
-      <c r="P17" s="25" t="s">
-        <v>744</v>
-      </c>
-      <c r="Q17" s="25" t="s">
-        <v>746</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A18" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B18" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="E18" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F18" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J18" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K18" s="25" t="s">
-        <v>622</v>
-      </c>
-      <c r="M18" s="25" t="s">
-        <v>789</v>
-      </c>
-      <c r="N18" s="25" t="s">
-        <v>626</v>
-      </c>
-      <c r="O18" s="25" t="s">
-        <v>577</v>
-      </c>
-      <c r="P18" s="25" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A19" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B19" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F19" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J19" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K19" s="25" t="s">
-        <v>622</v>
-      </c>
-      <c r="M19" s="25" t="s">
-        <v>788</v>
-      </c>
-      <c r="N19" s="25" t="s">
-        <v>626</v>
-      </c>
-      <c r="O19" s="25" t="s">
-        <v>578</v>
-      </c>
-      <c r="P19" s="25" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A20" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B20" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="E20" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F20" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J20" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K20" s="25" t="s">
-        <v>622</v>
-      </c>
-      <c r="M20" s="25" t="s">
-        <v>787</v>
-      </c>
-      <c r="N20" s="25" t="s">
-        <v>626</v>
-      </c>
-      <c r="O20" s="25" t="s">
-        <v>813</v>
-      </c>
-      <c r="P20" s="25" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C21" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="E21" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F21" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J21" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K21" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="L21" s="25" t="s">
-        <v>642</v>
-      </c>
-      <c r="N21" s="25" t="s">
-        <v>169</v>
-      </c>
-      <c r="O21" s="25" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B22" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="E22" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F22" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J22" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K22" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="L22" s="25" t="s">
-        <v>621</v>
-      </c>
-      <c r="R22" s="25" t="s">
-        <v>747</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A23" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B23" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C23" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="E23" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F23" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J23" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K23" s="25" t="s">
-        <v>814</v>
-      </c>
-      <c r="M23" s="25" t="s">
-        <v>785</v>
-      </c>
-      <c r="N23" s="25" t="s">
-        <v>161</v>
-      </c>
-      <c r="O23" s="25" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A24" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B24" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C24" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="E24" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F24" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J24" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K24" s="25" t="s">
-        <v>566</v>
-      </c>
-      <c r="L24" s="25" t="s">
-        <v>640</v>
-      </c>
-      <c r="N24" s="25" t="s">
-        <v>567</v>
-      </c>
-      <c r="O24" s="25" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A25" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B25" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C25" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E25" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F25" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J25" s="25" t="s">
-        <v>799</v>
-      </c>
-      <c r="K25" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="L25" s="26"/>
-      <c r="M25" s="26" t="s">
-        <v>768</v>
-      </c>
-      <c r="N25" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="O25" s="26" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A26" s="25" t="b">
-        <v>1</v>
-      </c>
-      <c r="B26" s="25" t="s">
-        <v>615</v>
-      </c>
-      <c r="C26" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="E26" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="F26" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="J26" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="K26" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="L26" s="25" t="s">
-        <v>644</v>
-      </c>
-      <c r="N26" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="O26" s="25" t="s">
-        <v>153</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S28">
-    <sortCondition ref="C1:C28"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T29">
+    <sortCondition ref="D1:D29"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -16430,7 +16487,7 @@
         <v>721</v>
       </c>
       <c r="L1" s="32" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="M1" s="32" t="s">
         <v>120</v>
@@ -16450,10 +16507,10 @@
         <v>146</v>
       </c>
       <c r="K2" s="40" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="L2" s="40" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="19" customHeight="1" x14ac:dyDescent="0.2">
@@ -16710,14 +16767,13 @@
     <col min="5" max="5" width="12.6640625" style="25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" style="25" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="25" customWidth="1"/>
-    <col min="9" max="9" width="13.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.6640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.5" style="25" customWidth="1"/>
+    <col min="8" max="8" width="21.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" style="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11" style="25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="18.5" style="25" customWidth="1"/>
     <col min="16" max="16" width="96.33203125" style="25" bestFit="1" customWidth="1"/>
     <col min="17" max="16384" width="10.83203125" style="25"/>
   </cols>
@@ -16745,28 +16801,28 @@
         <v>667</v>
       </c>
       <c r="H1" s="42" t="s">
-        <v>798</v>
-      </c>
-      <c r="I1" s="31" t="s">
-        <v>734</v>
+        <v>797</v>
+      </c>
+      <c r="I1" s="32" t="s">
+        <v>725</v>
       </c>
       <c r="J1" s="32" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="K1" s="32" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="L1" s="32" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="M1" s="32" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="N1" s="32" t="s">
-        <v>729</v>
+        <v>814</v>
       </c>
       <c r="O1" s="32" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="P1" s="32" t="s">
         <v>120</v>
@@ -16791,14 +16847,13 @@
       <c r="H2" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="I2" s="26"/>
+      <c r="I2" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J2" s="25" t="s">
-        <v>630</v>
+        <v>479</v>
       </c>
       <c r="K2" s="25" t="s">
-        <v>479</v>
-      </c>
-      <c r="L2" s="25" t="s">
         <v>639</v>
       </c>
     </row>
@@ -16818,17 +16873,16 @@
       <c r="H3" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="I3" s="26"/>
-      <c r="J3" s="25" t="s">
+      <c r="I3" s="25" t="s">
         <v>568</v>
       </c>
+      <c r="K3" s="25" t="s">
+        <v>662</v>
+      </c>
       <c r="L3" s="25" t="s">
-        <v>662</v>
+        <v>169</v>
       </c>
       <c r="M3" s="25" t="s">
-        <v>169</v>
-      </c>
-      <c r="N3" s="25" t="s">
         <v>156</v>
       </c>
     </row>
@@ -16851,14 +16905,13 @@
       <c r="H4" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="I4" s="26"/>
+      <c r="I4" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J4" s="25" t="s">
-        <v>630</v>
+        <v>499</v>
       </c>
       <c r="K4" s="25" t="s">
-        <v>499</v>
-      </c>
-      <c r="L4" s="25" t="s">
         <v>641</v>
       </c>
     </row>
@@ -16881,20 +16934,19 @@
       <c r="H5" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="I5" s="26"/>
+      <c r="I5" s="25" t="s">
+        <v>475</v>
+      </c>
       <c r="J5" s="25" t="s">
-        <v>475</v>
+        <v>630</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="L5" s="25" t="s">
-        <v>635</v>
+        <v>166</v>
       </c>
       <c r="M5" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="N5" s="25" t="s">
         <v>153</v>
       </c>
     </row>
@@ -16917,20 +16969,19 @@
       <c r="H6" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="I6" s="26"/>
+      <c r="I6" s="25" t="s">
+        <v>474</v>
+      </c>
       <c r="J6" s="25" t="s">
-        <v>474</v>
+        <v>630</v>
       </c>
       <c r="K6" s="25" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>634</v>
+        <v>155</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>155</v>
-      </c>
-      <c r="N6" s="25" t="s">
         <v>153</v>
       </c>
     </row>
@@ -16953,20 +17004,19 @@
       <c r="H7" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="I7" s="26"/>
+      <c r="I7" s="25" t="s">
+        <v>477</v>
+      </c>
       <c r="J7" s="25" t="s">
-        <v>477</v>
+        <v>630</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>630</v>
+        <v>637</v>
       </c>
       <c r="L7" s="25" t="s">
-        <v>637</v>
+        <v>166</v>
       </c>
       <c r="M7" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="N7" s="25" t="s">
         <v>153</v>
       </c>
     </row>
@@ -16989,20 +17039,19 @@
       <c r="H8" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I8" s="26"/>
+      <c r="I8" s="25" t="s">
+        <v>476</v>
+      </c>
       <c r="J8" s="25" t="s">
-        <v>476</v>
+        <v>630</v>
       </c>
       <c r="K8" s="25" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="L8" s="25" t="s">
-        <v>636</v>
+        <v>155</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>155</v>
-      </c>
-      <c r="N8" s="25" t="s">
         <v>153</v>
       </c>
     </row>
@@ -17025,22 +17074,18 @@
       <c r="H9" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="26"/>
-      <c r="J9" s="25" t="s">
+      <c r="I9" s="25" t="s">
         <v>478</v>
       </c>
+      <c r="K9" s="25" t="s">
+        <v>638</v>
+      </c>
       <c r="L9" s="25" t="s">
-        <v>638</v>
+        <v>799</v>
       </c>
       <c r="M9" s="25" t="s">
-        <v>800</v>
-      </c>
-      <c r="N9" s="25" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="I10" s="26"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="25" t="b">
@@ -17050,20 +17095,22 @@
         <v>615</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E11" s="25" t="s">
         <v>151</v>
       </c>
       <c r="H11" s="25" t="s">
+        <v>781</v>
+      </c>
+      <c r="J11" s="25" t="s">
+        <v>811</v>
+      </c>
+      <c r="K11" s="25" t="s">
+        <v>819</v>
+      </c>
+      <c r="N11" s="25" t="s">
         <v>782</v>
-      </c>
-      <c r="I11" s="26"/>
-      <c r="K11" s="25" t="s">
-        <v>812</v>
-      </c>
-      <c r="L11" s="25" t="s">
-        <v>783</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -17088,13 +17135,13 @@
       <c r="H13" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I13" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J13" s="25" t="s">
-        <v>630</v>
+        <v>423</v>
       </c>
       <c r="K13" s="25" t="s">
-        <v>423</v>
-      </c>
-      <c r="L13" s="25" t="s">
         <v>656</v>
       </c>
     </row>
@@ -17120,13 +17167,13 @@
       <c r="H14" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I14" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J14" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K14" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L14" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -17152,13 +17199,13 @@
       <c r="H15" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I15" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J15" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K15" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L15" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -17184,17 +17231,17 @@
       <c r="H16" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I16" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J16" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K16" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L16" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="b">
         <v>1</v>
       </c>
@@ -17216,14 +17263,14 @@
       <c r="H17" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I17" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J17" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="K17" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="b">
         <v>1</v>
       </c>
@@ -17245,17 +17292,17 @@
       <c r="H18" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I18" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J18" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K18" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L18" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="b">
         <v>1</v>
       </c>
@@ -17277,17 +17324,17 @@
       <c r="H19" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I19" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J19" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K19" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L19" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="b">
         <v>1</v>
       </c>
@@ -17309,17 +17356,17 @@
       <c r="H20" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I20" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J20" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K20" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L20" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="b">
         <v>1</v>
       </c>
@@ -17341,17 +17388,17 @@
       <c r="H21" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I21" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J21" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K21" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L21" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="b">
         <v>1</v>
       </c>
@@ -17373,17 +17420,17 @@
       <c r="H22" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I22" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J22" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K22" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L22" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="b">
         <v>1</v>
       </c>
@@ -17405,17 +17452,17 @@
       <c r="H23" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I23" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J23" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K23" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L23" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="b">
         <v>1</v>
       </c>
@@ -17437,17 +17484,17 @@
       <c r="H24" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I24" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J24" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K24" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L24" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="b">
         <v>1</v>
       </c>
@@ -17469,17 +17516,17 @@
       <c r="H25" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I25" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J25" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K25" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L25" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="25" t="b">
         <v>1</v>
       </c>
@@ -17501,17 +17548,17 @@
       <c r="H26" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I26" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J26" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K26" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L26" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="25" t="b">
         <v>1</v>
       </c>
@@ -17533,17 +17580,17 @@
       <c r="H27" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I27" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J27" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K27" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L27" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="25" t="b">
         <v>1</v>
       </c>
@@ -17565,17 +17612,17 @@
       <c r="H28" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I28" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J28" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K28" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L28" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="25" t="b">
         <v>1</v>
       </c>
@@ -17597,17 +17644,17 @@
       <c r="H29" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I29" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J29" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K29" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L29" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="25" t="b">
         <v>1</v>
       </c>
@@ -17629,17 +17676,17 @@
       <c r="H30" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I30" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J30" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K30" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L30" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="25" t="b">
         <v>1</v>
       </c>
@@ -17661,17 +17708,17 @@
       <c r="H31" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I31" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J31" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K31" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L31" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="25" t="b">
         <v>1</v>
       </c>
@@ -17693,17 +17740,17 @@
       <c r="H32" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I32" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J32" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K32" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L32" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="25" t="b">
         <v>1</v>
       </c>
@@ -17725,17 +17772,17 @@
       <c r="H33" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I33" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J33" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K33" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L33" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="25" t="b">
         <v>1</v>
       </c>
@@ -17757,17 +17804,17 @@
       <c r="H34" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I34" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J34" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K34" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L34" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="25" t="b">
         <v>1</v>
       </c>
@@ -17789,17 +17836,17 @@
       <c r="H35" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I35" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J35" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K35" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L35" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="25" t="b">
         <v>1</v>
       </c>
@@ -17821,20 +17868,20 @@
       <c r="H36" s="25" t="s">
         <v>29</v>
       </c>
+      <c r="I36" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J36" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K36" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L36" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D37" s="28"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="25" t="b">
         <v>1</v>
       </c>
@@ -17856,18 +17903,17 @@
       <c r="H38" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="I38" s="26"/>
+      <c r="I38" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J38" s="25" t="s">
-        <v>630</v>
+        <v>442</v>
       </c>
       <c r="K38" s="25" t="s">
-        <v>442</v>
-      </c>
-      <c r="L38" s="25" t="s">
         <v>657</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" s="25" t="b">
         <v>1</v>
       </c>
@@ -17889,17 +17935,17 @@
       <c r="H39" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I39" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J39" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K39" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L39" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="b">
         <v>1</v>
       </c>
@@ -17921,17 +17967,17 @@
       <c r="H40" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I40" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J40" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K40" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L40" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="b">
         <v>1</v>
       </c>
@@ -17953,17 +17999,17 @@
       <c r="H41" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I41" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J41" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K41" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L41" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="25" t="b">
         <v>1</v>
       </c>
@@ -17985,17 +18031,17 @@
       <c r="H42" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I42" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J42" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K42" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L42" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="25" t="b">
         <v>1</v>
       </c>
@@ -18017,17 +18063,17 @@
       <c r="H43" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I43" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J43" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K43" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L43" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="25" t="b">
         <v>1</v>
       </c>
@@ -18049,17 +18095,17 @@
       <c r="H44" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I44" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J44" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K44" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L44" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="25" t="b">
         <v>1</v>
       </c>
@@ -18081,17 +18127,17 @@
       <c r="H45" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I45" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J45" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K45" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L45" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="25" t="b">
         <v>1</v>
       </c>
@@ -18113,17 +18159,17 @@
       <c r="H46" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I46" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J46" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K46" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L46" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" s="25" t="b">
         <v>1</v>
       </c>
@@ -18145,17 +18191,17 @@
       <c r="H47" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I47" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J47" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K47" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L47" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="25" t="b">
         <v>1</v>
       </c>
@@ -18177,17 +18223,17 @@
       <c r="H48" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I48" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J48" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K48" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L48" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="25" t="b">
         <v>1</v>
       </c>
@@ -18209,17 +18255,17 @@
       <c r="H49" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I49" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J49" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K49" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L49" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="25" t="b">
         <v>1</v>
       </c>
@@ -18241,17 +18287,17 @@
       <c r="H50" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I50" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J50" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K50" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L50" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="25" t="b">
         <v>1</v>
       </c>
@@ -18273,17 +18319,17 @@
       <c r="H51" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I51" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J51" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K51" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L51" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" s="25" t="b">
         <v>1</v>
       </c>
@@ -18305,17 +18351,17 @@
       <c r="H52" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I52" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J52" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K52" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L52" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" s="25" t="b">
         <v>1</v>
       </c>
@@ -18337,17 +18383,17 @@
       <c r="H53" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I53" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J53" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K53" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L53" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" s="25" t="b">
         <v>1</v>
       </c>
@@ -18369,17 +18415,17 @@
       <c r="H54" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I54" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J54" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K54" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L54" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" s="25" t="b">
         <v>1</v>
       </c>
@@ -18401,17 +18447,17 @@
       <c r="H55" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I55" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J55" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K55" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L55" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" s="25" t="b">
         <v>1</v>
       </c>
@@ -18433,17 +18479,17 @@
       <c r="H56" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I56" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J56" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K56" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L56" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="25" t="b">
         <v>1</v>
       </c>
@@ -18465,17 +18511,17 @@
       <c r="H57" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I57" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J57" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K57" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L57" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="25" t="b">
         <v>1</v>
       </c>
@@ -18497,17 +18543,17 @@
       <c r="H58" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I58" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J58" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K58" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L58" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" s="25" t="b">
         <v>1</v>
       </c>
@@ -18529,17 +18575,17 @@
       <c r="H59" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I59" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J59" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K59" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L59" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="25" t="b">
         <v>1</v>
       </c>
@@ -18561,17 +18607,17 @@
       <c r="H60" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I60" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J60" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K60" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L60" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="25" t="b">
         <v>1</v>
       </c>
@@ -18593,17 +18639,17 @@
       <c r="H61" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I61" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J61" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K61" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L61" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="25" t="b">
         <v>1</v>
       </c>
@@ -18625,17 +18671,17 @@
       <c r="H62" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I62" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J62" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K62" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L62" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="25" t="b">
         <v>1</v>
       </c>
@@ -18657,17 +18703,17 @@
       <c r="H63" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I63" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J63" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K63" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L63" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="25" t="b">
         <v>1</v>
       </c>
@@ -18689,13 +18735,13 @@
       <c r="H64" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I64" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J64" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K64" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L64" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -18721,13 +18767,13 @@
       <c r="H65" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I65" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J65" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K65" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L65" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -18753,13 +18799,13 @@
       <c r="H66" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I66" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J66" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K66" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L66" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -18785,13 +18831,13 @@
       <c r="H67" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I67" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J67" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K67" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L67" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -18817,13 +18863,13 @@
       <c r="H68" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I68" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J68" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K68" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L68" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -18849,13 +18895,13 @@
       <c r="H69" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I69" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J69" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K69" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L69" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -18881,13 +18927,13 @@
       <c r="H70" s="25" t="s">
         <v>30</v>
       </c>
+      <c r="I70" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J70" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K70" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L70" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -18916,14 +18962,13 @@
       <c r="H72" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="I72" s="26"/>
+      <c r="I72" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J72" s="25" t="s">
-        <v>630</v>
+        <v>464</v>
       </c>
       <c r="K72" s="25" t="s">
-        <v>464</v>
-      </c>
-      <c r="L72" s="25" t="s">
         <v>660</v>
       </c>
     </row>
@@ -18949,13 +18994,13 @@
       <c r="H73" s="25" t="s">
         <v>41</v>
       </c>
+      <c r="I73" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J73" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K73" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L73" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -18981,13 +19026,13 @@
       <c r="H74" s="25" t="s">
         <v>41</v>
       </c>
+      <c r="I74" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J74" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K74" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L74" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -19013,13 +19058,13 @@
       <c r="H75" s="25" t="s">
         <v>41</v>
       </c>
+      <c r="I75" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J75" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K75" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L75" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -19045,13 +19090,13 @@
       <c r="H76" s="25" t="s">
         <v>41</v>
       </c>
+      <c r="I76" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J76" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K76" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L76" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -19077,13 +19122,13 @@
       <c r="H77" s="25" t="s">
         <v>41</v>
       </c>
+      <c r="I77" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J77" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K77" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L77" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -19109,13 +19154,13 @@
       <c r="H78" s="25" t="s">
         <v>41</v>
       </c>
+      <c r="I78" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J78" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K78" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L78" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -19144,21 +19189,20 @@
       <c r="H80" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="I80" s="26"/>
+      <c r="I80" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J80" s="25" t="s">
-        <v>630</v>
+        <v>502</v>
       </c>
       <c r="K80" s="25" t="s">
-        <v>502</v>
-      </c>
-      <c r="L80" s="25" t="s">
         <v>661</v>
       </c>
       <c r="O80" s="25" t="s">
-        <v>748</v>
-      </c>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" s="25" t="b">
         <v>1</v>
       </c>
@@ -19180,22 +19224,20 @@
       <c r="H81" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="I81" s="26"/>
+      <c r="I81" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J81" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K81" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L81" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D82" s="28"/>
-      <c r="I82" s="26"/>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" s="25" t="b">
         <v>1</v>
       </c>
@@ -19214,18 +19256,17 @@
       <c r="H83" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="I83" s="26"/>
+      <c r="I83" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J83" s="25" t="s">
-        <v>630</v>
+        <v>481</v>
       </c>
       <c r="K83" s="25" t="s">
-        <v>481</v>
-      </c>
-      <c r="L83" s="25" t="s">
         <v>659</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" s="25" t="b">
         <v>1</v>
       </c>
@@ -19247,17 +19288,17 @@
       <c r="H84" s="25" t="s">
         <v>38</v>
       </c>
+      <c r="I84" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J84" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K84" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L84" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" s="25" t="b">
         <v>1</v>
       </c>
@@ -19279,17 +19320,17 @@
       <c r="H85" s="25" t="s">
         <v>38</v>
       </c>
+      <c r="I85" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J85" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K85" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L85" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" s="25" t="b">
         <v>1</v>
       </c>
@@ -19311,17 +19352,17 @@
       <c r="H86" s="25" t="s">
         <v>38</v>
       </c>
+      <c r="I86" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J86" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K86" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L86" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" s="25" t="b">
         <v>1</v>
       </c>
@@ -19343,17 +19384,17 @@
       <c r="H87" s="25" t="s">
         <v>38</v>
       </c>
+      <c r="I87" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J87" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K87" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L87" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" s="25" t="b">
         <v>1</v>
       </c>
@@ -19375,17 +19416,17 @@
       <c r="H88" s="25" t="s">
         <v>38</v>
       </c>
+      <c r="I88" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J88" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K88" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L88" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" s="25" t="b">
         <v>1</v>
       </c>
@@ -19407,20 +19448,20 @@
       <c r="H89" s="25" t="s">
         <v>38</v>
       </c>
+      <c r="I89" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J89" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K89" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L89" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D90" s="28"/>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="b">
         <v>1</v>
       </c>
@@ -19439,18 +19480,17 @@
       <c r="H91" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="I91" s="26"/>
+      <c r="I91" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J91" s="25" t="s">
-        <v>630</v>
+        <v>480</v>
       </c>
       <c r="K91" s="25" t="s">
-        <v>480</v>
-      </c>
-      <c r="L91" s="25" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" s="25" t="b">
         <v>1</v>
       </c>
@@ -19472,17 +19512,17 @@
       <c r="H92" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I92" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J92" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K92" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L92" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="b">
         <v>1</v>
       </c>
@@ -19504,17 +19544,17 @@
       <c r="H93" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I93" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J93" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K93" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L93" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" s="25" t="b">
         <v>1</v>
       </c>
@@ -19536,17 +19576,17 @@
       <c r="H94" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I94" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J94" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K94" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L94" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" s="25" t="b">
         <v>1</v>
       </c>
@@ -19568,17 +19608,17 @@
       <c r="H95" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I95" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J95" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K95" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L95" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" s="25" t="b">
         <v>1</v>
       </c>
@@ -19600,17 +19640,17 @@
       <c r="H96" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I96" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J96" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K96" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L96" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" s="25" t="b">
         <v>1</v>
       </c>
@@ -19632,17 +19672,17 @@
       <c r="H97" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I97" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J97" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K97" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L97" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" s="25" t="b">
         <v>1</v>
       </c>
@@ -19664,17 +19704,17 @@
       <c r="H98" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I98" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J98" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K98" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L98" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" s="25" t="b">
         <v>1</v>
       </c>
@@ -19696,17 +19736,17 @@
       <c r="H99" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I99" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J99" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K99" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L99" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" s="25" t="b">
         <v>1</v>
       </c>
@@ -19728,17 +19768,17 @@
       <c r="H100" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I100" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J100" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K100" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L100" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" s="25" t="b">
         <v>1</v>
       </c>
@@ -19760,17 +19800,17 @@
       <c r="H101" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I101" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J101" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K101" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L101" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" s="25" t="b">
         <v>1</v>
       </c>
@@ -19792,17 +19832,17 @@
       <c r="H102" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I102" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J102" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K102" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L102" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" s="25" t="b">
         <v>1</v>
       </c>
@@ -19824,17 +19864,17 @@
       <c r="H103" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I103" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J103" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K103" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L103" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" s="25" t="b">
         <v>1</v>
       </c>
@@ -19856,17 +19896,17 @@
       <c r="H104" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I104" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J104" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K104" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L104" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" s="25" t="b">
         <v>1</v>
       </c>
@@ -19888,17 +19928,17 @@
       <c r="H105" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I105" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J105" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K105" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L105" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" s="25" t="b">
         <v>1</v>
       </c>
@@ -19920,20 +19960,20 @@
       <c r="H106" s="25" t="s">
         <v>37</v>
       </c>
+      <c r="I106" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J106" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K106" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L106" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D107" s="28"/>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" s="25" t="b">
         <v>1</v>
       </c>
@@ -19955,17 +19995,17 @@
       <c r="H108" s="25" t="s">
         <v>28</v>
       </c>
+      <c r="I108" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J108" s="25" t="s">
-        <v>630</v>
+        <v>418</v>
       </c>
       <c r="K108" s="25" t="s">
-        <v>418</v>
-      </c>
-      <c r="L108" s="25" t="s">
         <v>655</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" s="25" t="b">
         <v>1</v>
       </c>
@@ -19987,17 +20027,17 @@
       <c r="H109" s="25" t="s">
         <v>28</v>
       </c>
+      <c r="I109" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J109" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K109" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L109" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" s="25" t="b">
         <v>1</v>
       </c>
@@ -20019,17 +20059,17 @@
       <c r="H110" s="25" t="s">
         <v>28</v>
       </c>
+      <c r="I110" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J110" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K110" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L110" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111" s="25" t="b">
         <v>1</v>
       </c>
@@ -20051,17 +20091,17 @@
       <c r="H111" s="25" t="s">
         <v>28</v>
       </c>
+      <c r="I111" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J111" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K111" s="25" t="s">
         <v>630</v>
       </c>
-      <c r="L111" s="25" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" s="25" t="b">
         <v>1</v>
       </c>
@@ -20080,13 +20120,13 @@
       <c r="H112" s="25" t="s">
         <v>28</v>
       </c>
+      <c r="I112" s="25" t="s">
+        <v>630</v>
+      </c>
       <c r="J112" s="25" t="s">
         <v>630</v>
       </c>
       <c r="K112" s="25" t="s">
-        <v>630</v>
-      </c>
-      <c r="L112" s="25" t="s">
         <v>630</v>
       </c>
     </row>
@@ -20143,37 +20183,37 @@
         <v>667</v>
       </c>
       <c r="H1" s="31" t="s">
+        <v>771</v>
+      </c>
+      <c r="I1" s="32" t="s">
         <v>772</v>
       </c>
-      <c r="I1" s="32" t="s">
+      <c r="J1" s="32" t="s">
         <v>773</v>
       </c>
-      <c r="J1" s="32" t="s">
+      <c r="K1" s="32" t="s">
         <v>774</v>
       </c>
-      <c r="K1" s="32" t="s">
+      <c r="L1" s="23" t="s">
+        <v>795</v>
+      </c>
+      <c r="M1" s="32" t="s">
         <v>775</v>
       </c>
-      <c r="L1" s="23" t="s">
+      <c r="N1" s="32" t="s">
+        <v>776</v>
+      </c>
+      <c r="O1" s="32" t="s">
+        <v>777</v>
+      </c>
+      <c r="P1" s="23" t="s">
         <v>796</v>
       </c>
-      <c r="M1" s="32" t="s">
-        <v>776</v>
-      </c>
-      <c r="N1" s="32" t="s">
-        <v>777</v>
-      </c>
-      <c r="O1" s="32" t="s">
-        <v>778</v>
-      </c>
-      <c r="P1" s="23" t="s">
-        <v>797</v>
-      </c>
       <c r="Q1" s="32" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="R1" s="31" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
@@ -20199,7 +20239,7 @@
         <v>40</v>
       </c>
       <c r="M2" s="25" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="O2" s="25" t="s">
         <v>655</v>
@@ -20208,7 +20248,7 @@
         <v>28</v>
       </c>
       <c r="Q2" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -20234,7 +20274,7 @@
         <v>28</v>
       </c>
       <c r="M3" s="25" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="O3" s="25" t="s">
         <v>634</v>
@@ -20243,7 +20283,7 @@
         <v>31</v>
       </c>
       <c r="Q3" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
@@ -20269,7 +20309,7 @@
         <v>32</v>
       </c>
       <c r="M4" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O4" s="25" t="s">
         <v>634</v>
@@ -20278,7 +20318,7 @@
         <v>31</v>
       </c>
       <c r="Q4" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
@@ -20304,7 +20344,7 @@
         <v>31</v>
       </c>
       <c r="M5" s="25" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="O5" s="25" t="s">
         <v>656</v>
@@ -20313,7 +20353,7 @@
         <v>29</v>
       </c>
       <c r="Q5" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
@@ -20339,7 +20379,7 @@
         <v>35</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O6" s="25" t="s">
         <v>656</v>
@@ -20348,7 +20388,7 @@
         <v>29</v>
       </c>
       <c r="Q6" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
@@ -20374,7 +20414,7 @@
         <v>29</v>
       </c>
       <c r="M7" s="25" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="O7" s="25" t="s">
         <v>636</v>
@@ -20383,7 +20423,7 @@
         <v>33</v>
       </c>
       <c r="Q7" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
@@ -20409,7 +20449,7 @@
         <v>34</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O8" s="25" t="s">
         <v>636</v>
@@ -20418,7 +20458,7 @@
         <v>33</v>
       </c>
       <c r="Q8" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
@@ -20444,7 +20484,7 @@
         <v>33</v>
       </c>
       <c r="M9" s="25" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="O9" s="25" t="s">
         <v>657</v>
@@ -20453,7 +20493,7 @@
         <v>30</v>
       </c>
       <c r="Q9" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
@@ -20479,7 +20519,7 @@
         <v>36</v>
       </c>
       <c r="M10" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O10" s="25" t="s">
         <v>657</v>
@@ -20488,7 +20528,7 @@
         <v>30</v>
       </c>
       <c r="Q10" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
@@ -20514,7 +20554,7 @@
         <v>37</v>
       </c>
       <c r="M11" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O11" s="25" t="s">
         <v>639</v>
@@ -20523,7 +20563,7 @@
         <v>36</v>
       </c>
       <c r="Q11" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
@@ -20549,7 +20589,7 @@
         <v>38</v>
       </c>
       <c r="M12" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O12" s="25" t="s">
         <v>639</v>
@@ -20558,7 +20598,7 @@
         <v>36</v>
       </c>
       <c r="Q12" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
@@ -20584,7 +20624,7 @@
         <v>30</v>
       </c>
       <c r="M13" s="25" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="O13" s="25" t="s">
         <v>660</v>
@@ -20593,7 +20633,7 @@
         <v>41</v>
       </c>
       <c r="Q13" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
@@ -20619,7 +20659,7 @@
         <v>42</v>
       </c>
       <c r="M14" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O14" s="25" t="s">
         <v>660</v>
@@ -20628,7 +20668,7 @@
         <v>41</v>
       </c>
       <c r="Q14" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
@@ -20639,7 +20679,7 @@
         <v>615</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E15" s="25" t="s">
         <v>710</v>
@@ -20648,13 +20688,13 @@
         <v>688</v>
       </c>
       <c r="K15" s="25" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="L15" s="25" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="M15" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O15" s="25" t="s">
         <v>660</v>
@@ -20663,7 +20703,7 @@
         <v>41</v>
       </c>
       <c r="Q15" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
@@ -20689,7 +20729,7 @@
         <v>43</v>
       </c>
       <c r="M16" s="25" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="O16" s="25" t="s">
         <v>660</v>
@@ -20698,7 +20738,7 @@
         <v>41</v>
       </c>
       <c r="Q16" s="25" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
   </sheetData>
@@ -20886,7 +20926,7 @@
         <v>395</v>
       </c>
       <c r="I11" s="25" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -21343,7 +21383,7 @@
         <v>395</v>
       </c>
       <c r="I46" s="25" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
@@ -21669,7 +21709,7 @@
         <v>289</v>
       </c>
       <c r="I70" s="25" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
@@ -22663,7 +22703,7 @@
         <v>360</v>
       </c>
       <c r="I141" s="25" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.2">
@@ -22677,7 +22717,7 @@
         <v>361</v>
       </c>
       <c r="I142" s="25" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.2">
@@ -22691,7 +22731,7 @@
         <v>362</v>
       </c>
       <c r="I143" s="25" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.2">
@@ -22705,7 +22745,7 @@
         <v>363</v>
       </c>
       <c r="I144" s="25" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.2">
@@ -22719,7 +22759,7 @@
         <v>364</v>
       </c>
       <c r="I145" s="25" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.2">
@@ -22733,7 +22773,7 @@
         <v>365</v>
       </c>
       <c r="I146" s="25" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.2">
@@ -22747,7 +22787,7 @@
         <v>366</v>
       </c>
       <c r="I147" s="25" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.2">
@@ -23142,7 +23182,7 @@
         <v>258</v>
       </c>
       <c r="I176" s="25" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.2">
@@ -23156,7 +23196,7 @@
         <v>259</v>
       </c>
       <c r="I177" s="25" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.2">
@@ -23360,7 +23400,7 @@
         <v>1</v>
       </c>
       <c r="D193" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E193" s="27" t="s">
         <v>84</v>
@@ -23374,7 +23414,7 @@
         <v>1</v>
       </c>
       <c r="D194" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E194" s="27" t="s">
         <v>85</v>
@@ -23388,7 +23428,7 @@
         <v>1</v>
       </c>
       <c r="D195" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E195" s="41" t="s">
         <v>86</v>
@@ -23402,7 +23442,7 @@
         <v>1</v>
       </c>
       <c r="D196" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E196" s="41" t="s">
         <v>87</v>
@@ -23416,7 +23456,7 @@
         <v>1</v>
       </c>
       <c r="D197" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E197" s="41" t="s">
         <v>88</v>
@@ -23430,7 +23470,7 @@
         <v>1</v>
       </c>
       <c r="D198" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E198" s="28" t="s">
         <v>89</v>
@@ -23444,7 +23484,7 @@
         <v>1</v>
       </c>
       <c r="D199" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E199" s="28" t="s">
         <v>90</v>
@@ -23458,7 +23498,7 @@
         <v>1</v>
       </c>
       <c r="D200" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E200" s="27" t="s">
         <v>91</v>
@@ -23472,7 +23512,7 @@
         <v>1</v>
       </c>
       <c r="D201" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E201" s="27" t="s">
         <v>92</v>
@@ -23486,7 +23526,7 @@
         <v>1</v>
       </c>
       <c r="D202" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E202" s="28" t="s">
         <v>93</v>
@@ -23500,7 +23540,7 @@
         <v>1</v>
       </c>
       <c r="D203" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E203" s="28" t="s">
         <v>94</v>
@@ -23514,7 +23554,7 @@
         <v>1</v>
       </c>
       <c r="D204" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E204" s="28" t="s">
         <v>95</v>
@@ -23528,7 +23568,7 @@
         <v>1</v>
       </c>
       <c r="D205" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E205" s="28" t="s">
         <v>96</v>
@@ -23542,7 +23582,7 @@
         <v>1</v>
       </c>
       <c r="D206" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E206" s="28" t="s">
         <v>97</v>
@@ -23556,7 +23596,7 @@
         <v>1</v>
       </c>
       <c r="D207" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E207" s="28" t="s">
         <v>98</v>
@@ -23570,7 +23610,7 @@
         <v>1</v>
       </c>
       <c r="D208" s="25" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E208" s="28" t="s">
         <v>99</v>

</xml_diff>

<commit_message>
Fixed inhibition_method typo in wide_protocolSteps
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18857A13-B1CB-E84E-BE47-72AF98C007BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8BA9DB-380B-524D-A3A5-A3B4A0585CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" activeTab="1" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" activeTab="3" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2921" uniqueCount="820">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2922" uniqueCount="820">
   <si>
     <t>Reporter</t>
   </si>
@@ -2561,7 +2561,7 @@
     <t>selectors</t>
   </si>
   <si>
-    <t>null</t>
+    <t>case(((inhibition_method == "") + (inhibition_method == None), ""), (True, "null"))</t>
   </si>
 </sst>
 </file>
@@ -16757,7 +16757,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDC6A21B-0669-0743-9D12-F41DCA15CA4A}">
-  <dimension ref="A1:P112"/>
+  <dimension ref="A1:Q112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="25" bestFit="1" customWidth="1"/>
@@ -16771,14 +16771,15 @@
     <col min="9" max="9" width="15.6640625" style="25" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.5" style="25" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="22.83203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11" style="25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="18.5" style="25" customWidth="1"/>
-    <col min="16" max="16" width="96.33203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="10.83203125" style="25"/>
+    <col min="12" max="12" width="22.83203125" style="25" customWidth="1"/>
+    <col min="13" max="13" width="11" style="25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.5" style="25" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="18.5" style="25" customWidth="1"/>
+    <col min="17" max="17" width="96.33203125" style="25" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="10.83203125" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="31" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="31" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="31" t="s">
         <v>651</v>
       </c>
@@ -16813,22 +16814,25 @@
         <v>727</v>
       </c>
       <c r="L1" s="32" t="s">
+        <v>734</v>
+      </c>
+      <c r="M1" s="32" t="s">
         <v>728</v>
       </c>
-      <c r="M1" s="32" t="s">
+      <c r="N1" s="32" t="s">
         <v>729</v>
       </c>
-      <c r="N1" s="32" t="s">
+      <c r="O1" s="32" t="s">
         <v>814</v>
       </c>
-      <c r="O1" s="32" t="s">
+      <c r="P1" s="32" t="s">
         <v>751</v>
       </c>
-      <c r="P1" s="32" t="s">
+      <c r="Q1" s="32" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="b">
         <v>1</v>
       </c>
@@ -16857,7 +16861,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="b">
         <v>1</v>
       </c>
@@ -16879,14 +16883,14 @@
       <c r="K3" s="25" t="s">
         <v>662</v>
       </c>
-      <c r="L3" s="25" t="s">
+      <c r="M3" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="M3" s="25" t="s">
+      <c r="N3" s="25" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="b">
         <v>1</v>
       </c>
@@ -16915,7 +16919,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="b">
         <v>1</v>
       </c>
@@ -16943,14 +16947,14 @@
       <c r="K5" s="25" t="s">
         <v>635</v>
       </c>
-      <c r="L5" s="25" t="s">
+      <c r="M5" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="M5" s="25" t="s">
+      <c r="N5" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="b">
         <v>1</v>
       </c>
@@ -16978,14 +16982,14 @@
       <c r="K6" s="25" t="s">
         <v>634</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="M6" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="M6" s="25" t="s">
+      <c r="N6" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="b">
         <v>1</v>
       </c>
@@ -17013,14 +17017,14 @@
       <c r="K7" s="25" t="s">
         <v>637</v>
       </c>
-      <c r="L7" s="25" t="s">
+      <c r="M7" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="M7" s="25" t="s">
+      <c r="N7" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="b">
         <v>1</v>
       </c>
@@ -17048,14 +17052,14 @@
       <c r="K8" s="25" t="s">
         <v>636</v>
       </c>
-      <c r="L8" s="25" t="s">
+      <c r="M8" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="M8" s="25" t="s">
+      <c r="N8" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="b">
         <v>1</v>
       </c>
@@ -17080,14 +17084,14 @@
       <c r="K9" s="25" t="s">
         <v>638</v>
       </c>
-      <c r="L9" s="25" t="s">
+      <c r="M9" s="25" t="s">
         <v>799</v>
       </c>
-      <c r="M9" s="25" t="s">
+      <c r="N9" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" s="25" t="b">
         <v>1</v>
       </c>
@@ -17106,14 +17110,14 @@
       <c r="J11" s="25" t="s">
         <v>811</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="L11" s="25" t="s">
         <v>819</v>
       </c>
-      <c r="N11" s="25" t="s">
+      <c r="O11" s="25" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="b">
         <v>1</v>
       </c>
@@ -17145,7 +17149,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="b">
         <v>1</v>
       </c>
@@ -17177,7 +17181,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="b">
         <v>1</v>
       </c>
@@ -17209,7 +17213,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="b">
         <v>1</v>
       </c>
@@ -18745,7 +18749,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65" s="25" t="b">
         <v>1</v>
       </c>
@@ -18777,7 +18781,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66" s="25" t="b">
         <v>1</v>
       </c>
@@ -18809,7 +18813,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67" s="25" t="b">
         <v>1</v>
       </c>
@@ -18841,7 +18845,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A68" s="25" t="b">
         <v>1</v>
       </c>
@@ -18873,7 +18877,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A69" s="25" t="b">
         <v>1</v>
       </c>
@@ -18905,7 +18909,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A70" s="25" t="b">
         <v>1</v>
       </c>
@@ -18937,10 +18941,10 @@
         <v>630</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D71" s="30"/>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A72" s="25" t="b">
         <v>1</v>
       </c>
@@ -18972,7 +18976,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A73" s="25" t="b">
         <v>1</v>
       </c>
@@ -19004,7 +19008,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A74" s="25" t="b">
         <v>1</v>
       </c>
@@ -19036,7 +19040,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A75" s="25" t="b">
         <v>1</v>
       </c>
@@ -19068,7 +19072,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A76" s="25" t="b">
         <v>1</v>
       </c>
@@ -19100,7 +19104,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A77" s="25" t="b">
         <v>1</v>
       </c>
@@ -19132,7 +19136,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A78" s="25" t="b">
         <v>1</v>
       </c>
@@ -19164,10 +19168,10 @@
         <v>630</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D79" s="28"/>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A80" s="25" t="b">
         <v>1</v>
       </c>
@@ -19198,7 +19202,7 @@
       <c r="K80" s="25" t="s">
         <v>661</v>
       </c>
-      <c r="O80" s="25" t="s">
+      <c r="P80" s="25" t="s">
         <v>747</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Change mapping of population_served -> sites.popServe to population_served -> measures table
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/nwss_to_odm_v2_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8BA9DB-380B-524D-A3A5-A3B4A0585CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB8F50E-EBDD-E543-853E-4B4BFB98E95B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20860" activeTab="3" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="40960" windowHeight="20760" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2922" uniqueCount="820">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2930" uniqueCount="822">
   <si>
     <t>Reporter</t>
   </si>
@@ -2562,6 +2562,12 @@
   </si>
   <si>
     <t>case(((inhibition_method == "") + (inhibition_method == None), ""), (True, "null"))</t>
+  </si>
+  <si>
+    <t>pop</t>
+  </si>
+  <si>
+    <t>peeps</t>
   </si>
 </sst>
 </file>
@@ -2857,6 +2863,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="parts"/>
@@ -15309,7 +15316,7 @@
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" s="25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B79" s="25" t="s">
         <v>615</v>
@@ -15497,7 +15504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39AC7DD-3F73-2C47-925D-21E5B4EBE6FC}">
-  <dimension ref="A1:T28"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="25"/>
@@ -16421,6 +16428,35 @@
         <v>161</v>
       </c>
       <c r="P28" s="25" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A30" s="25" t="b">
+        <v>1</v>
+      </c>
+      <c r="B30" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D30" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="K30" s="25" t="s">
+        <v>820</v>
+      </c>
+      <c r="L30" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="M30" s="25" t="s">
+        <v>681</v>
+      </c>
+      <c r="O30" s="25" t="s">
+        <v>821</v>
+      </c>
+      <c r="P30" s="25" t="s">
         <v>156</v>
       </c>
     </row>
@@ -23803,7 +23839,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>1</v>

</xml_diff>